<commit_message>
Add surname dictionary alert (486 surnames, Levenshtein distance check)
</commit_message>
<xml_diff>
--- a/step3-validation-check.xlsx
+++ b/step3-validation-check.xlsx
@@ -2862,44 +2862,44 @@
       <c r="H63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="inlineStr">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>適格性質問</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>質問⑨</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>63</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>Yes時詳細入力</t>
         </is>
       </c>
-      <c r="E64" s="3" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>渡航日/目的/期間の入力欄</t>
         </is>
       </c>
-      <c r="F64" s="3" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>未実装</t>
         </is>
       </c>
-      <c r="G64" s="3" t="inlineStr">
-        <is>
-          <t>❌</t>
-        </is>
-      </c>
-      <c r="H64" s="3" t="inlineStr">
-        <is>
-          <t>Yes回答時のサブ質問なし</t>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>省略（「はい」回答時はESTA認証不可のためサブ質問不要）</t>
         </is>
       </c>
     </row>

</xml_diff>